<commit_message>
Updated data about minimized solutions
</commit_message>
<xml_diff>
--- a/data_analysis/analysis_selected_solutions.xlsx
+++ b/data_analysis/analysis_selected_solutions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dados\Dafny\TESTDAFNY110\data_analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C3729A8-E5A1-46D9-A5AE-A0FFDBED66FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18B6EEB2-6D94-4432-BEFF-E0FBA7E4F7B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{AD00872A-3429-4154-B9D8-B04F44A65181}"/>
   </bookViews>
@@ -1074,7 +1074,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1095,6 +1095,7 @@
     <xf numFmtId="10" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4290,11 +4291,11 @@
       </c>
       <c r="G9">
         <f>IFERROR(VLOOKUP(C9,locs_minimized!A:B,2,0),F9)</f>
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="I9">
         <f t="shared" si="1"/>
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.45">
@@ -4450,11 +4451,11 @@
       </c>
       <c r="G14">
         <f>IFERROR(VLOOKUP(C14,locs_minimized!A:B,2,0),F14)</f>
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I14">
         <f t="shared" si="1"/>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.45">
@@ -4482,11 +4483,11 @@
       </c>
       <c r="G15">
         <f>IFERROR(VLOOKUP(C15,locs_minimized!A:B,2,0),F15)</f>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I15">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.45">
@@ -4514,11 +4515,11 @@
       </c>
       <c r="G16">
         <f>IFERROR(VLOOKUP(C16,locs_minimized!A:B,2,0),F16)</f>
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="I16">
         <f t="shared" si="1"/>
-        <v>30</v>
+        <v>19</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.45">
@@ -4578,11 +4579,11 @@
       </c>
       <c r="G18">
         <f>IFERROR(VLOOKUP(C18,locs_minimized!A:B,2,0),F18)</f>
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="I18">
         <f t="shared" si="1"/>
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.45">
@@ -4610,11 +4611,11 @@
       </c>
       <c r="G19">
         <f>IFERROR(VLOOKUP(C19,locs_minimized!A:B,2,0),F19)</f>
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I19">
         <f t="shared" si="1"/>
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.45">
@@ -4642,11 +4643,11 @@
       </c>
       <c r="G20">
         <f>IFERROR(VLOOKUP(C20,locs_minimized!A:B,2,0),F20)</f>
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="I20">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.45">
@@ -4674,11 +4675,11 @@
       </c>
       <c r="G21">
         <f>IFERROR(VLOOKUP(C21,locs_minimized!A:B,2,0),F21)</f>
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="I21">
         <f t="shared" si="1"/>
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.45">
@@ -4898,11 +4899,11 @@
       </c>
       <c r="G28">
         <f>IFERROR(VLOOKUP(C28,locs_minimized!A:B,2,0),F28)</f>
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="I28">
         <f t="shared" si="1"/>
-        <v>13</v>
+        <v>19</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.45">
@@ -5058,11 +5059,11 @@
       </c>
       <c r="G33">
         <f>IFERROR(VLOOKUP(C33,locs_minimized!A:B,2,0),F33)</f>
-        <v>69</v>
+        <v>46</v>
       </c>
       <c r="I33">
         <f t="shared" si="1"/>
-        <v>39</v>
+        <v>16</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.45">
@@ -5250,11 +5251,11 @@
       </c>
       <c r="G39">
         <f>IFERROR(VLOOKUP(C39,locs_minimized!A:B,2,0),F39)</f>
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="I39">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.45">
@@ -5506,11 +5507,11 @@
       </c>
       <c r="G47">
         <f>IFERROR(VLOOKUP(C47,locs_minimized!A:B,2,0),F47)</f>
-        <v>61</v>
+        <v>49</v>
       </c>
       <c r="I47">
         <f t="shared" si="1"/>
-        <v>19</v>
+        <v>7</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.45">
@@ -5954,11 +5955,11 @@
       </c>
       <c r="G61">
         <f>IFERROR(VLOOKUP(C61,locs_minimized!A:B,2,0),F61)</f>
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="I61">
         <f t="shared" si="1"/>
-        <v>-8</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.45">
@@ -6114,11 +6115,11 @@
       </c>
       <c r="G66">
         <f>IFERROR(VLOOKUP(C66,locs_minimized!A:B,2,0),F66)</f>
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="I66">
         <f t="shared" si="1"/>
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.45">
@@ -6146,11 +6147,11 @@
       </c>
       <c r="G67">
         <f>IFERROR(VLOOKUP(C67,locs_minimized!A:B,2,0),F67)</f>
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="I67">
         <f t="shared" ref="I67:I110" si="3">G67-D67</f>
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.45">
@@ -6178,11 +6179,11 @@
       </c>
       <c r="G68">
         <f>IFERROR(VLOOKUP(C68,locs_minimized!A:B,2,0),F68)</f>
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I68">
         <f t="shared" si="3"/>
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.45">
@@ -6466,11 +6467,11 @@
       </c>
       <c r="G77">
         <f>IFERROR(VLOOKUP(C77,locs_minimized!A:B,2,0),F77)</f>
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I77">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.45">
@@ -6690,11 +6691,11 @@
       </c>
       <c r="G84">
         <f>IFERROR(VLOOKUP(C84,locs_minimized!A:B,2,0),F84)</f>
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="I84">
         <f t="shared" si="3"/>
-        <v>52</v>
+        <v>46</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.45">
@@ -6882,11 +6883,11 @@
       </c>
       <c r="G90">
         <f>IFERROR(VLOOKUP(C90,locs_minimized!A:B,2,0),F90)</f>
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="I90">
         <f t="shared" si="3"/>
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.45">
@@ -7330,11 +7331,11 @@
       </c>
       <c r="G104">
         <f>IFERROR(VLOOKUP(C104,locs_minimized!A:B,2,0),F104)</f>
-        <v>60</v>
+        <v>44</v>
       </c>
       <c r="I104">
         <f t="shared" si="3"/>
-        <v>30</v>
+        <v>14</v>
       </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.45">
@@ -7394,11 +7395,11 @@
       </c>
       <c r="G106">
         <f>IFERROR(VLOOKUP(C106,locs_minimized!A:B,2,0),F106)</f>
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="I106">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>-10</v>
       </c>
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.45">
@@ -7490,11 +7491,11 @@
       </c>
       <c r="G109">
         <f>IFERROR(VLOOKUP(C109,locs_minimized!A:B,2,0),F109)</f>
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="I109">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.45">
@@ -7515,11 +7516,11 @@
       </c>
       <c r="G110">
         <f t="shared" si="4"/>
-        <v>3809</v>
+        <v>3751</v>
       </c>
       <c r="I110">
         <f t="shared" si="3"/>
-        <v>412</v>
+        <v>354</v>
       </c>
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.45">
@@ -7532,13 +7533,13 @@
       </c>
       <c r="G111" s="5">
         <f>G110/D110-1</f>
-        <v>0.12128348542831913</v>
+        <v>0.10420959670297325</v>
       </c>
     </row>
     <row r="112" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="G112">
-        <f>(G110-E110)/(F110-E110)</f>
-        <v>0.44090177133655395</v>
+      <c r="G112" s="10">
+        <f>1-(G110-E110)/(F110-E110)</f>
+        <v>0.57777777777777772</v>
       </c>
     </row>
   </sheetData>
@@ -9721,7 +9722,7 @@
         <v>241</v>
       </c>
       <c r="B6">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.45">
@@ -9753,7 +9754,7 @@
         <v>244</v>
       </c>
       <c r="B10">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.45">
@@ -9761,7 +9762,7 @@
         <v>245</v>
       </c>
       <c r="B11">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.45">
@@ -9769,7 +9770,7 @@
         <v>246</v>
       </c>
       <c r="B12">
-        <v>75</v>
+        <v>64</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.45">
@@ -9785,7 +9786,7 @@
         <v>248</v>
       </c>
       <c r="B14">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.45">
@@ -9793,7 +9794,7 @@
         <v>249</v>
       </c>
       <c r="B15">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.45">
@@ -9801,7 +9802,7 @@
         <v>250</v>
       </c>
       <c r="B16">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.45">
@@ -9809,7 +9810,7 @@
         <v>317</v>
       </c>
       <c r="B17">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.45">
@@ -9857,7 +9858,7 @@
         <v>256</v>
       </c>
       <c r="B23">
-        <v>59</v>
+        <v>65</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.45">
@@ -9889,7 +9890,7 @@
         <v>260</v>
       </c>
       <c r="B27">
-        <v>69</v>
+        <v>46</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.45">
@@ -9905,7 +9906,7 @@
         <v>262</v>
       </c>
       <c r="B29">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.45">
@@ -9953,7 +9954,7 @@
         <v>268</v>
       </c>
       <c r="B35">
-        <v>61</v>
+        <v>49</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.45">
@@ -10009,7 +10010,7 @@
         <v>275</v>
       </c>
       <c r="B42">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.45">
@@ -10025,7 +10026,7 @@
         <v>276</v>
       </c>
       <c r="B44">
-        <v>33</v>
+        <v>28</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.45">
@@ -10033,7 +10034,7 @@
         <v>277</v>
       </c>
       <c r="B45">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.45">
@@ -10041,7 +10042,7 @@
         <v>278</v>
       </c>
       <c r="B46">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.45">
@@ -10097,7 +10098,7 @@
         <v>285</v>
       </c>
       <c r="B53">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.45">
@@ -10137,7 +10138,7 @@
         <v>290</v>
       </c>
       <c r="B58">
-        <v>100</v>
+        <v>94</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.45">
@@ -10153,7 +10154,7 @@
         <v>292</v>
       </c>
       <c r="B60">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.45">
@@ -10249,7 +10250,7 @@
         <v>303</v>
       </c>
       <c r="B72">
-        <v>60</v>
+        <v>44</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.45">
@@ -10257,7 +10258,7 @@
         <v>304</v>
       </c>
       <c r="B73">
-        <v>36</v>
+        <v>25</v>
       </c>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.45">
@@ -10281,7 +10282,7 @@
         <v>307</v>
       </c>
       <c r="B76">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated simplify.py script and results
</commit_message>
<xml_diff>
--- a/data_analysis/analysis_selected_solutions.xlsx
+++ b/data_analysis/analysis_selected_solutions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dados\Dafny\TESTDAFNY110\data_analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18B6EEB2-6D94-4432-BEFF-E0FBA7E4F7B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C58C879-4270-471F-9538-4523557D1E8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{AD00872A-3429-4154-B9D8-B04F44A65181}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="982" uniqueCount="323">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1015" uniqueCount="323">
   <si>
     <t>Filename</t>
   </si>
@@ -5507,11 +5507,11 @@
       </c>
       <c r="G47">
         <f>IFERROR(VLOOKUP(C47,locs_minimized!A:B,2,0),F47)</f>
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="I47">
         <f t="shared" si="1"/>
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.45">
@@ -7516,11 +7516,11 @@
       </c>
       <c r="G110">
         <f t="shared" si="4"/>
-        <v>3751</v>
+        <v>3747</v>
       </c>
       <c r="I110">
         <f t="shared" si="3"/>
-        <v>354</v>
+        <v>350</v>
       </c>
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.45">
@@ -7533,13 +7533,13 @@
       </c>
       <c r="G111" s="5">
         <f>G110/D110-1</f>
-        <v>0.10420959670297325</v>
+        <v>0.10303208713570799</v>
       </c>
     </row>
     <row r="112" spans="1:9" x14ac:dyDescent="0.45">
       <c r="G112" s="10">
         <f>1-(G110-E110)/(F110-E110)</f>
-        <v>0.57777777777777772</v>
+        <v>0.57906602254428341</v>
       </c>
     </row>
   </sheetData>
@@ -9671,7 +9671,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E69E5DE-7812-4896-B0F1-C7271BDE67E5}">
-  <dimension ref="A1:B76"/>
+  <dimension ref="A1:B109"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="32.6640625" bestFit="1" customWidth="1"/>
@@ -9954,7 +9954,7 @@
         <v>268</v>
       </c>
       <c r="B35">
-        <v>49</v>
+        <v>45</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.45">
@@ -10283,6 +10283,270 @@
       </c>
       <c r="B76">
         <v>34</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A77" t="s">
+        <v>199</v>
+      </c>
+      <c r="B77">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A78" t="s">
+        <v>200</v>
+      </c>
+      <c r="B78">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A79" t="s">
+        <v>202</v>
+      </c>
+      <c r="B79">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A80" t="s">
+        <v>203</v>
+      </c>
+      <c r="B80">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A81" t="s">
+        <v>204</v>
+      </c>
+      <c r="B81">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A82" t="s">
+        <v>205</v>
+      </c>
+      <c r="B82">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A83" t="s">
+        <v>201</v>
+      </c>
+      <c r="B83">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A84" t="s">
+        <v>206</v>
+      </c>
+      <c r="B84">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A85" t="s">
+        <v>207</v>
+      </c>
+      <c r="B85">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A86" t="s">
+        <v>208</v>
+      </c>
+      <c r="B86">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A87" t="s">
+        <v>209</v>
+      </c>
+      <c r="B87">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A88" t="s">
+        <v>210</v>
+      </c>
+      <c r="B88">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A89" t="s">
+        <v>211</v>
+      </c>
+      <c r="B89">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A90" t="s">
+        <v>212</v>
+      </c>
+      <c r="B90">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A91" t="s">
+        <v>213</v>
+      </c>
+      <c r="B91">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A92" t="s">
+        <v>214</v>
+      </c>
+      <c r="B92">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A93" t="s">
+        <v>215</v>
+      </c>
+      <c r="B93">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A94" t="s">
+        <v>216</v>
+      </c>
+      <c r="B94">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A95" t="s">
+        <v>217</v>
+      </c>
+      <c r="B95">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A96" t="s">
+        <v>218</v>
+      </c>
+      <c r="B96">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A97" t="s">
+        <v>219</v>
+      </c>
+      <c r="B97">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A98" t="s">
+        <v>220</v>
+      </c>
+      <c r="B98">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A99" t="s">
+        <v>221</v>
+      </c>
+      <c r="B99">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A100" t="s">
+        <v>222</v>
+      </c>
+      <c r="B100">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A101" t="s">
+        <v>223</v>
+      </c>
+      <c r="B101">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A102" t="s">
+        <v>224</v>
+      </c>
+      <c r="B102">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A103" t="s">
+        <v>226</v>
+      </c>
+      <c r="B103">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A104" t="s">
+        <v>227</v>
+      </c>
+      <c r="B104">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A105" t="s">
+        <v>228</v>
+      </c>
+      <c r="B105">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A106" t="s">
+        <v>229</v>
+      </c>
+      <c r="B106">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A107" t="s">
+        <v>230</v>
+      </c>
+      <c r="B107">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A108" t="s">
+        <v>225</v>
+      </c>
+      <c r="B108">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A109" t="s">
+        <v>231</v>
+      </c>
+      <c r="B109">
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>